<commit_message>
fix(financeiro): grupos da aba Renda sem "Total mensal:" na extração
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/lib/finance/import/fixtures/mini.xlsx
+++ b/src/lib/finance/import/fixtures/mini.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="35">
   <si>
     <t>JAN</t>
   </si>
@@ -608,9 +608,6 @@
       <c r="B7" t="s">
         <v>18</v>
       </c>
-      <c r="G7" t="s">
-        <v>14</v>
-      </c>
       <c r="J7">
         <f>SUM(J1:J2)</f>
         <v>1.5</v>

</xml_diff>